<commit_message>
Fix Excel import: case-insensitive column matching and updated sample files
</commit_message>
<xml_diff>
--- a/super-admin-paneli/Ornek_Exceller/Akademisyenler_Ornek.xlsx
+++ b/super-admin-paneli/Ornek_Exceller/Akademisyenler_Ornek.xlsx
@@ -397,26 +397,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Unvan</v>
+        <v>unvan</v>
       </c>
       <c r="B1" t="str">
-        <v>Ad</v>
+        <v>ad</v>
       </c>
       <c r="C1" t="str">
-        <v>Soyad</v>
+        <v>soyad</v>
       </c>
       <c r="D1" t="str">
-        <v>Eposta</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Kullanici_Adi</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Sifre</v>
+        <v>eposta</v>
       </c>
     </row>
     <row r="2">
@@ -432,12 +426,6 @@
       <c r="D2" t="str">
         <v>ahmet.yilmaz@uni.edu.tr</v>
       </c>
-      <c r="E2" t="str">
-        <v>ahmet.yilmaz</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Sifre123!</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -452,16 +440,52 @@
       <c r="D3" t="str">
         <v>ayse.kaya@uni.edu.tr</v>
       </c>
-      <c r="E3" t="str">
-        <v>ayse.kaya</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Sifre123!</v>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Dr. Öğr. Üyesi</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Mehmet</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Demir</v>
+      </c>
+      <c r="D4" t="str">
+        <v>mehmet.demir@uni.edu.tr</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fatma</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Çelik</v>
+      </c>
+      <c r="D5" t="str">
+        <v>fatma.celik@uni.edu.tr</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Ali</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Öztürk</v>
+      </c>
+      <c r="D6" t="str">
+        <v>ali.ozturk@uni.edu.tr</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>